<commit_message>
Last status , everything completed
</commit_message>
<xml_diff>
--- a/project3/submission_files/GroupMembers.xlsx
+++ b/project3/submission_files/GroupMembers.xlsx
@@ -3,9 +3,9 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D371B42-D1C7-420B-8A79-7BD67B98A512}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{286EA11F-4073-40CD-BA9D-CCDE025659D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2652" yWindow="2652" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,10 +34,10 @@
     <t>StudentID</t>
   </si>
   <si>
-    <t>Name1 Surname1</t>
+    <t>Hüseyin Teke</t>
   </si>
   <si>
-    <t>Name2 Surname2</t>
+    <t>Aysun Dilara Doğan</t>
   </si>
 </sst>
 </file>
@@ -379,7 +379,7 @@
         <v>23727</v>
       </c>
       <c r="B2">
-        <v>111111111</v>
+        <v>150230089</v>
       </c>
       <c r="C2" t="s">
         <v>3</v>
@@ -387,10 +387,10 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>23728</v>
+        <v>23727</v>
       </c>
       <c r="B3">
-        <v>222222222</v>
+        <v>150230040</v>
       </c>
       <c r="C3" t="s">
         <v>4</v>

</xml_diff>